<commit_message>
feat: add TC-INVENTORY-011 test case
</commit_message>
<xml_diff>
--- a/test-cases/Test_Cases_SwagLabs.xlsx
+++ b/test-cases/Test_Cases_SwagLabs.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="106">
   <si>
     <t xml:space="preserve">TEST CASE DOCUMENT — Swag Labs (SauceDemo)</t>
   </si>
@@ -375,6 +375,22 @@
   </si>
   <si>
     <t xml:space="preserve">TC-INVENTORY-011</t>
+  </si>
+  <si>
+    <t xml:space="preserve">URL Manipulation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aplikasi dapat diakses di browser, user belum login</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Buka browser
+2. Akses langsung url https://www.saucedemo.com/inventory.html tanpa login</t>
+  </si>
+  <si>
+    <t xml:space="preserve">User diredirect ke halaman login dan muncul pesan "You can only access '/inventory.html' when you are logged in."</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Security test</t>
   </si>
   <si>
     <t xml:space="preserve">TEST SUMMARY — Login Module</t>
@@ -1693,7 +1709,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
         <v>95</v>
       </c>
@@ -1701,28 +1717,28 @@
         <v>46</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>88</v>
+        <v>96</v>
       </c>
       <c r="D14" s="8" t="s">
-        <v>89</v>
+        <v>97</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>90</v>
+        <v>98</v>
       </c>
       <c r="F14" s="8" t="s">
-        <v>91</v>
+        <v>99</v>
       </c>
       <c r="G14" s="8" t="s">
-        <v>92</v>
-      </c>
-      <c r="H14" s="12" t="s">
-        <v>93</v>
+        <v>99</v>
+      </c>
+      <c r="H14" s="6" t="s">
+        <v>18</v>
       </c>
       <c r="I14" s="7" t="s">
         <v>19</v>
       </c>
       <c r="J14" s="5" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
     </row>
   </sheetData>
@@ -1758,13 +1774,13 @@
   <sheetData>
     <row r="1" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="13" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="B1" s="13"/>
     </row>
     <row r="2" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="14" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="B2" s="15" t="n">
         <f aca="false">COUNTA('TC - Login'!A4:A92)</f>
@@ -1773,19 +1789,19 @@
     </row>
     <row r="3" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="16" t="s">
-        <v>98</v>
+        <v>103</v>
       </c>
       <c r="B3" s="17"/>
     </row>
     <row r="4" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="14" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="B4" s="15"/>
     </row>
     <row r="5" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="16" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="B5" s="17" t="n">
         <f aca="false">B2-B3-B4</f>

</xml_diff>